<commit_message>
Updated excel data method
</commit_message>
<xml_diff>
--- a/project_code/src/main/resources/TestDataSheet.xlsx
+++ b/project_code/src/main/resources/TestDataSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2110883_cognizant_com/Documents/Desktop/ninjaWeb_Automation/ninjaTutirial_CompleteProject/project_code/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_F25DC773A252ABDACC104896619C6DB05ADE5907" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C20D733-F7EF-4C3F-8F46-9EABEDB3F513}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="11_F25DC773A252ABDACC104896619C6DB05ADE5907" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67F35EDA-2098-4EAA-84DF-31B89DF4853F}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
   <si>
     <t>First Name</t>
   </si>
@@ -58,13 +58,82 @@
   </si>
   <si>
     <t>New User</t>
+  </si>
+  <si>
+    <t>Pavan</t>
+  </si>
+  <si>
+    <t>Hiware</t>
+  </si>
+  <si>
+    <t>pavanhiware11@gmail.com</t>
+  </si>
+  <si>
+    <t>Valid User</t>
+  </si>
+  <si>
+    <t>Hiware12345</t>
+  </si>
+  <si>
+    <t>Invalid User</t>
+  </si>
+  <si>
+    <t>New Password</t>
+  </si>
+  <si>
+    <t>Hiware123</t>
+  </si>
+  <si>
+    <t>Used</t>
+  </si>
+  <si>
+    <t>Saicharn</t>
+  </si>
+  <si>
+    <t>Diware</t>
+  </si>
+  <si>
+    <t>saiDiware11@gamil.com</t>
+  </si>
+  <si>
+    <t>Sai@123</t>
+  </si>
+  <si>
+    <t>Rushu</t>
+  </si>
+  <si>
+    <t>Wagh</t>
+  </si>
+  <si>
+    <t>rushWag12@gamil.com</t>
+  </si>
+  <si>
+    <t>Rush@321</t>
+  </si>
+  <si>
+    <t>New Userr</t>
+  </si>
+  <si>
+    <t>Ram</t>
+  </si>
+  <si>
+    <t>Madhav</t>
+  </si>
+  <si>
+    <t>ramMadhav22@gamil.com</t>
+  </si>
+  <si>
+    <t>Ram@22</t>
+  </si>
+  <si>
+    <t>New Userrr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -76,6 +145,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -123,11 +198,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -409,10 +485,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultColWidth="12.875" defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -429,10 +505,13 @@
         <v>5</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -448,14 +527,127 @@
       <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2"/>
+      <c r="G2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3">
+        <v>7218688193</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>7218688193</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5">
+        <v>9881343521</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6">
+        <v>7832124521</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7">
+        <v>7421342167</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{C9AA45D3-763C-49D8-8615-A269442DA2D2}"/>
     <hyperlink ref="E2" r:id="rId2" xr:uid="{D299E41E-0D4E-4B2E-B18E-81CE9669E643}"/>
+    <hyperlink ref="C3" r:id="rId3" xr:uid="{61631589-3655-490D-BACA-5AEC9D8923F7}"/>
+    <hyperlink ref="C4" r:id="rId4" xr:uid="{85C08829-7DF8-4628-9440-33B11E57217A}"/>
+    <hyperlink ref="C5" r:id="rId5" xr:uid="{F04DAC94-7373-4A61-903D-830C4109381B}"/>
+    <hyperlink ref="E5" r:id="rId6" xr:uid="{E7079178-30D0-4E88-913D-0A8DC63AD648}"/>
+    <hyperlink ref="C6" r:id="rId7" xr:uid="{D0CA259A-AD69-4D42-A8DB-95C0303B053E}"/>
+    <hyperlink ref="E6" r:id="rId8" xr:uid="{85BEA752-2220-475C-B642-E7AF71D237D8}"/>
+    <hyperlink ref="C7" r:id="rId9" xr:uid="{1306871C-8457-4907-A830-5A38986B646B}"/>
+    <hyperlink ref="E7" r:id="rId10" xr:uid="{8C061893-AD93-47CB-965E-60BCA326C316}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>